<commit_message>
Laminas regeneradas (regeneracion completa del 2026-10-04), piramides 2018-2024, empates nombrados (#191) (graficos_regionales_piramide)
</commit_message>
<xml_diff>
--- a/output/graficos_regionales_piramide/plot_comunal_piramide_2018_biobio.xlsx
+++ b/output/graficos_regionales_piramide/plot_comunal_piramide_2018_biobio.xlsx
@@ -141,13 +141,13 @@
     <t xml:space="preserve">Curanilahue</t>
   </si>
   <si>
-    <t xml:space="preserve">Los Alamos</t>
+    <t xml:space="preserve">Los Álamos</t>
   </si>
   <si>
     <t xml:space="preserve">Tirúa</t>
   </si>
   <si>
-    <t xml:space="preserve">Los Angeles</t>
+    <t xml:space="preserve">Los Ángeles</t>
   </si>
   <si>
     <t xml:space="preserve">Antuco</t>
@@ -198,7 +198,7 @@
     <t xml:space="preserve">Fecha de creación</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-09-30 15:39</t>
+    <t xml:space="preserve">2026-10-05 21:04</t>
   </si>
   <si>
     <t xml:space="preserve">Fuente</t>

</xml_diff>